<commit_message>
docs: revise IJCCS manuscript after review
Addresses all review points: single-resource scope in title and aims,
threshold-free P/R/F1 (Table 6), stage-1 selection vs. conditional stage-2
accuracy (Table 7), Encounter absorption recomputed with the definition
catalogue for both models (Table 9), explicit evaluation procedure with a
worked example, confirmatory test family, honest pre-registration statement,
quoted prompts, and corrected model-gap figures. Figure 1 now marks gold
correspondences as illustration. The annotation kit gains a resource-level
agreement sheet. All new numbers come from cached model outputs
(revision_analyses.py, 0 new LLM calls). Point-by-point response in
paper/ijccs/tanggapan_reviewer.md; kappa, author details and repository URL
are still pending.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/annotation/anotasi_kedua.xlsx
+++ b/annotation/anotasi_kedua.xlsx
@@ -8,18 +8,19 @@
   </bookViews>
   <sheets>
     <sheet name="Petunjuk" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Anotasi" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="FHIR_Patient" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="FHIR_Practitioner" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="FHIR_Location" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="FHIR_Encounter" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="FHIR_Condition" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="FHIR_MedicationRequest" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="FHIR_Medication" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="FHIR_Organization" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="FHIR_ServiceRequest" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="FHIR_DiagnosticReport" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet name="FHIR_Observation" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet name="Resource" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Anotasi" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="FHIR_Patient" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="FHIR_Practitioner" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="FHIR_Location" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="FHIR_Encounter" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="FHIR_Condition" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="FHIR_MedicationRequest" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="FHIR_Medication" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="FHIR_Organization" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="FHIR_ServiceRequest" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="FHIR_DiagnosticReport" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet name="FHIR_Observation" sheetId="14" state="visible" r:id="rId14"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -461,6 +462,7 @@
 5. Nomor kunjungan/rawat (no_rawat, no_redis, idRekamMedis) pada tabel selain kunjungan itu sendiri adalah referensi -&gt; "encounter", bukan "identifier".
 6. Tabel tanda vital: kolom tekanan darah -&gt; component.value[x] (1:1), vital lain -&gt; component.value[x] (n:1).
 7. Kolom tarif/harga dan kolom audit aplikasi (created_at, user input) -&gt; tidak ada, kecuali jelas padanannya.
+Di sheet "Resource", nyatakan apakah Anda setuju dengan resource FHIR yang ditetapkan untuk tiap tabel; bila tidak, tulis resource alternatif. Kolom pada sheet "Anotasi" tetap diisi terhadap resource yang ditetapkan.
 Jangan melihat file GT lain dan jangan menjalankan model. Perkiraan waktu ±4 jam; boleh dicicil.
 </t>
         </is>
@@ -472,6 +474,262 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C14"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="32" customWidth="1" min="1" max="1"/>
+    <col width="90" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>elemen</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>tipe</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>deskripsi (FHIR short)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>identifier</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Identifier</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Business identifier for this medication</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>CodeableConcept</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Codes that identify this medication</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>status</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>active | inactive | entered-in-error</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>manufacturer</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Reference</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Manufacturer of the item</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>form</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>CodeableConcept</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>powder | tablets | capsule +</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>amount</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Ratio</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Amount of drug in package</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>ingredient</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>BackboneElement</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Active or inactive ingredient</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>ingredient.item[x]</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>CodeableConcept|Reference</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>The actual ingredient or content</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>ingredient.isActive</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>boolean</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Active ingredient indicator</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>ingredient.strength</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Ratio</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Quantity of ingredient present</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>batch</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>BackboneElement</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Details about packaged medications</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>batch.lotNumber</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Identifier assigned to batch</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>batch.expirationDate</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>dateTime</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>When batch will expire</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -744,7 +1002,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1340,7 +1598,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1715,7 +1973,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2325,6 +2583,1127 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F60"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="34" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="40" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>pasangan</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>tabel sumber</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>resource yang ditetapkan</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Setuju? (ya/tidak)</t>
+        </is>
+      </c>
+      <c r="E1" s="2" t="inlineStr">
+        <is>
+          <t>Resource alternatif</t>
+        </is>
+      </c>
+      <c r="F1" s="2" t="inlineStr">
+        <is>
+          <t>Catatan</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>E01</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>khanza__pasien</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Patient</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="n"/>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>E02</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>khanza__dokter</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Practitioner</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="n"/>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>E03</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>khanza__pegawai</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Practitioner</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="n"/>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>E04</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>khanza__poliklinik</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Location</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="n"/>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>E05</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>khanza__reg_periksa</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Encounter</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="n"/>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>E06</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>khanza__diagnosa_pasien</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Condition</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="n"/>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>E07</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>khanza__resep_obat</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>MedicationRequest</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="n"/>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>E08</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>khanza__resep_dokter</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>MedicationRequest</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="n"/>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>E09</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>khanza__databarang</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Medication</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="n"/>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>E10</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>khanza__kamar_inap</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Encounter</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>E11</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>khanza__penjab</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Organization</t>
+        </is>
+      </c>
+      <c r="D12" s="3" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>E12</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>khanza__rujuk</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>ServiceRequest</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>E13</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>khanza__periksa_lab</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>DiagnosticReport</t>
+        </is>
+      </c>
+      <c r="D14" s="3" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>E14</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>khanza__detail_periksa_lab</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Observation</t>
+        </is>
+      </c>
+      <c r="D15" s="3" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>E20</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>opensid__tweb_penduduk</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Patient</t>
+        </is>
+      </c>
+      <c r="D16" s="3" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>E29</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>khanza__pasien_mati</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Patient</t>
+        </is>
+      </c>
+      <c r="D17" s="3" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>E30</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>khanza__pasien_corona</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Patient</t>
+        </is>
+      </c>
+      <c r="D18" s="3" t="n"/>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>E31</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>khanza__petugas</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Practitioner</t>
+        </is>
+      </c>
+      <c r="D19" s="3" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>E32</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>khanza__perusahaan_pasien</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Organization</t>
+        </is>
+      </c>
+      <c r="D20" s="3" t="n"/>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>E33</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>khanza__industrifarmasi</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Organization</t>
+        </is>
+      </c>
+      <c r="D21" s="3" t="n"/>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>E34</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>khanza__datasuplier</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Organization</t>
+        </is>
+      </c>
+      <c r="D22" s="3" t="n"/>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>E35</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>khanza__bangsal</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Location</t>
+        </is>
+      </c>
+      <c r="D23" s="3" t="n"/>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>E36</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>khanza__kamar</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Location</t>
+        </is>
+      </c>
+      <c r="D24" s="3" t="n"/>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>E37</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>khanza__ruang_ok</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Location</t>
+        </is>
+      </c>
+      <c r="D25" s="3" t="n"/>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>E38</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>khanza__dpjp_ranap</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Encounter</t>
+        </is>
+      </c>
+      <c r="D26" s="3" t="n"/>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>E39</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>khanza__resume_pasien</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Condition</t>
+        </is>
+      </c>
+      <c r="D27" s="3" t="n"/>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>E40</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>khanza__pemeriksaan_ralan</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Observation</t>
+        </is>
+      </c>
+      <c r="D28" s="3" t="n"/>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>E41</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>khanza__pemeriksaan_ranap</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Observation</t>
+        </is>
+      </c>
+      <c r="D29" s="3" t="n"/>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>E42</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>khanza__catatan_observasi_igd</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Observation</t>
+        </is>
+      </c>
+      <c r="D30" s="3" t="n"/>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>E43</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>khanza__catatan_observasi_ranap</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Observation</t>
+        </is>
+      </c>
+      <c r="D31" s="3" t="n"/>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>E44</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>khanza__data_triase_igd</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Observation</t>
+        </is>
+      </c>
+      <c r="D32" s="3" t="n"/>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>E45</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>khanza__skrining_gizi</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Observation</t>
+        </is>
+      </c>
+      <c r="D33" s="3" t="n"/>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>E46</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>khanza__skrining_hipertensi</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Observation</t>
+        </is>
+      </c>
+      <c r="D34" s="3" t="n"/>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>E47</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>khanza__resep_dokter_racikan</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>MedicationRequest</t>
+        </is>
+      </c>
+      <c r="D35" s="3" t="n"/>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>E48</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>khanza__resep_pulang</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>MedicationRequest</t>
+        </is>
+      </c>
+      <c r="D36" s="3" t="n"/>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>E49</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>khanza__periksa_radiologi</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>DiagnosticReport</t>
+        </is>
+      </c>
+      <c r="D37" s="3" t="n"/>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>E50</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>khanza__hasil_radiologi</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>DiagnosticReport</t>
+        </is>
+      </c>
+      <c r="D38" s="3" t="n"/>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>E51</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>khanza__permintaan_lab</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>ServiceRequest</t>
+        </is>
+      </c>
+      <c r="D39" s="3" t="n"/>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>E52</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>khanza__permintaan_radiologi</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>ServiceRequest</t>
+        </is>
+      </c>
+      <c r="D40" s="3" t="n"/>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>E53</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>khanza__rujukan_internal_poli</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>ServiceRequest</t>
+        </is>
+      </c>
+      <c r="D41" s="3" t="n"/>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>E54</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>khanza__rujuk_masuk</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>ServiceRequest</t>
+        </is>
+      </c>
+      <c r="D42" s="3" t="n"/>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>C01</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>rmpuskesmas__tb_pasien</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>Patient</t>
+        </is>
+      </c>
+      <c r="D43" s="3" t="n"/>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>C02</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>rmpuskesmas__tb_rekam_medis</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>Encounter</t>
+        </is>
+      </c>
+      <c r="D44" s="3" t="n"/>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>C03</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>rmpuskesmas__tb_rujuk</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>ServiceRequest</t>
+        </is>
+      </c>
+      <c r="D45" s="3" t="n"/>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>C04</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>rmpuskesmas__tb_resep</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>MedicationRequest</t>
+        </is>
+      </c>
+      <c r="D46" s="3" t="n"/>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>C05</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>rmpuskesmas__tb_dokter</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>Practitioner</t>
+        </is>
+      </c>
+      <c r="D47" s="3" t="n"/>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>C06</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>sipuskesmas__polis</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>Location</t>
+        </is>
+      </c>
+      <c r="D48" s="3" t="n"/>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>C07</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>sipuskesmas__tenaga_kesehatans</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>Practitioner</t>
+        </is>
+      </c>
+      <c r="D49" s="3" t="n"/>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>C08</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>sipuskesmas__antrians</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>Encounter</t>
+        </is>
+      </c>
+      <c r="D50" s="3" t="n"/>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>C09</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>cirekammedis__dokter</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>Practitioner</t>
+        </is>
+      </c>
+      <c r="D51" s="3" t="n"/>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>C10</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>cirekammedis__obat</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>Medication</t>
+        </is>
+      </c>
+      <c r="D52" s="3" t="n"/>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>C11</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>cirekammedis__pasien</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>Patient</t>
+        </is>
+      </c>
+      <c r="D53" s="3" t="n"/>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>C12</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>cirekammedis__poliklinik</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>Location</t>
+        </is>
+      </c>
+      <c r="D54" s="3" t="n"/>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>C13</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>cirekammedis__rekam_medis</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>Encounter</t>
+        </is>
+      </c>
+      <c r="D55" s="3" t="n"/>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>C14</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>cirekammedis__rm_obat</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>MedicationRequest</t>
+        </is>
+      </c>
+      <c r="D56" s="3" t="n"/>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>C15</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>sipograf__t_anak</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>Patient</t>
+        </is>
+      </c>
+      <c r="D57" s="3" t="n"/>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>C16</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>sipograf__t_penimbangan</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>Observation</t>
+        </is>
+      </c>
+      <c r="D58" s="3" t="n"/>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>C17</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>epuskesmas__obat</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>Medication</t>
+        </is>
+      </c>
+      <c r="D59" s="3" t="n"/>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>C18</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>opensid__posyandu</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>Organization</t>
+        </is>
+      </c>
+      <c r="D60" s="3" t="n"/>
+    </row>
+  </sheetData>
+  <dataValidations count="1">
+    <dataValidation sqref="D2 D3 D4 D5 D6 D7 D8 D9 D10 D11 D12 D13 D14 D15 D16 D17 D18 D19 D20 D21 D22 D23 D24 D25 D26 D27 D28 D29 D30 D31 D32 D33 D34 D35 D36 D37 D38 D39 D40 D41 D42 D43 D44 D45 D46 D47 D48 D49 D50 D51 D52 D53 D54 D55 D56 D57 D58 D59 D60" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"ya,tidak"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -23105,7 +24484,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -23582,7 +24961,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -23855,7 +25234,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -24298,7 +25677,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -25115,7 +26494,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -25524,7 +26903,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -26288,260 +27667,4 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:C14"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="32" customWidth="1" min="1" max="1"/>
-    <col width="90" customWidth="1" min="3" max="3"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>elemen</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>tipe</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>deskripsi (FHIR short)</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>identifier</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>Identifier</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>Business identifier for this medication</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>code</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>CodeableConcept</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>Codes that identify this medication</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>status</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>code</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>active | inactive | entered-in-error</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>manufacturer</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>Reference</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>Manufacturer of the item</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>form</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>CodeableConcept</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>powder | tablets | capsule +</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>amount</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>Ratio</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>Amount of drug in package</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>ingredient</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>BackboneElement</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>Active or inactive ingredient</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>ingredient.item[x]</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>CodeableConcept|Reference</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>The actual ingredient or content</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>ingredient.isActive</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>boolean</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>Active ingredient indicator</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>ingredient.strength</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>Ratio</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>Quantity of ingredient present</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>batch</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>BackboneElement</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>Details about packaged medications</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>batch.lotNumber</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>string</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>Identifier assigned to batch</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>batch.expirationDate</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>dateTime</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>When batch will expire</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
docs: third-round revision of IJCCS manuscript
Redesigns the second annotation as two phases so resource agreement is
measured between independent choices (phase 1 hides the assigned resource),
and reports four agreement measures. Adds a formal definition of the three
evaluation policies, labels the GLM deployment-strict confirm18 result as
exploratory, softens the human-confirmation conclusion, limits the embedding
claim to the classifiers tested, states exact model versions (Ollama digests,
API model id and access date), adds a dated post-review addendum to the
pre-registration, and keeps "R@|GT|" from wrapping in tables and captions.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/annotation/anotasi_kedua.xlsx
+++ b/annotation/anotasi_kedua.xlsx
@@ -8,19 +8,18 @@
   </bookViews>
   <sheets>
     <sheet name="Petunjuk" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Resource" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Anotasi" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="FHIR_Patient" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="FHIR_Practitioner" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="FHIR_Location" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="FHIR_Encounter" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="FHIR_Condition" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="FHIR_MedicationRequest" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="FHIR_Medication" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="FHIR_Organization" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="FHIR_ServiceRequest" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet name="FHIR_DiagnosticReport" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet name="FHIR_Observation" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet name="Anotasi" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="FHIR_Patient" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="FHIR_Practitioner" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="FHIR_Location" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="FHIR_Encounter" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="FHIR_Condition" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="FHIR_MedicationRequest" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="FHIR_Medication" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="FHIR_Organization" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="FHIR_ServiceRequest" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="FHIR_DiagnosticReport" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="FHIR_Observation" sheetId="13" state="visible" r:id="rId13"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -462,7 +461,7 @@
 5. Nomor kunjungan/rawat (no_rawat, no_redis, idRekamMedis) pada tabel selain kunjungan itu sendiri adalah referensi -&gt; "encounter", bukan "identifier".
 6. Tabel tanda vital: kolom tekanan darah -&gt; component.value[x] (1:1), vital lain -&gt; component.value[x] (n:1).
 7. Kolom tarif/harga dan kolom audit aplikasi (created_at, user input) -&gt; tidak ada, kecuali jelas padanannya.
-Di sheet "Resource", nyatakan apakah Anda setuju dengan resource FHIR yang ditetapkan untuk tiap tabel; bila tidak, tulis resource alternatif. Kolom pada sheet "Anotasi" tetap diisi terhadap resource yang ditetapkan.
+Tahap 2: file ini dibuka SETELAH tahap 1 (pemilihan resource) dikirim. Kolom di sheet "Anotasi" diisi terhadap resource yang ditetapkan di kolom "resource target".
 Jangan melihat file GT lain dan jangan menjalankan model. Perkiraan waktu ±4 jam; boleh dicicil.
 </t>
         </is>
@@ -474,262 +473,6 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:C14"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="32" customWidth="1" min="1" max="1"/>
-    <col width="90" customWidth="1" min="3" max="3"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>elemen</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>tipe</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>deskripsi (FHIR short)</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>identifier</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>Identifier</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>Business identifier for this medication</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>code</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>CodeableConcept</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>Codes that identify this medication</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>status</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>code</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>active | inactive | entered-in-error</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>manufacturer</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>Reference</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>Manufacturer of the item</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>form</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>CodeableConcept</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>powder | tablets | capsule +</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>amount</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>Ratio</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>Amount of drug in package</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>ingredient</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>BackboneElement</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>Active or inactive ingredient</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>ingredient.item[x]</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>CodeableConcept|Reference</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>The actual ingredient or content</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>ingredient.isActive</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>boolean</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>Active ingredient indicator</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>ingredient.strength</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>Ratio</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>Quantity of ingredient present</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>batch</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>BackboneElement</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>Details about packaged medications</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>batch.lotNumber</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>string</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>Identifier assigned to batch</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>batch.expirationDate</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>dateTime</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>When batch will expire</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1002,7 +745,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1598,7 +1341,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1973,7 +1716,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2583,1127 +2326,6 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:F60"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="10" customWidth="1" min="1" max="1"/>
-    <col width="34" customWidth="1" min="2" max="2"/>
-    <col width="22" customWidth="1" min="3" max="3"/>
-    <col width="18" customWidth="1" min="4" max="4"/>
-    <col width="22" customWidth="1" min="5" max="5"/>
-    <col width="40" customWidth="1" min="6" max="6"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="2" t="inlineStr">
-        <is>
-          <t>pasangan</t>
-        </is>
-      </c>
-      <c r="B1" s="2" t="inlineStr">
-        <is>
-          <t>tabel sumber</t>
-        </is>
-      </c>
-      <c r="C1" s="2" t="inlineStr">
-        <is>
-          <t>resource yang ditetapkan</t>
-        </is>
-      </c>
-      <c r="D1" s="2" t="inlineStr">
-        <is>
-          <t>Setuju? (ya/tidak)</t>
-        </is>
-      </c>
-      <c r="E1" s="2" t="inlineStr">
-        <is>
-          <t>Resource alternatif</t>
-        </is>
-      </c>
-      <c r="F1" s="2" t="inlineStr">
-        <is>
-          <t>Catatan</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>E01</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>khanza__pasien</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>Patient</t>
-        </is>
-      </c>
-      <c r="D2" s="3" t="n"/>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>E02</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>khanza__dokter</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>Practitioner</t>
-        </is>
-      </c>
-      <c r="D3" s="3" t="n"/>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>E03</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>khanza__pegawai</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>Practitioner</t>
-        </is>
-      </c>
-      <c r="D4" s="3" t="n"/>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>E04</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>khanza__poliklinik</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>Location</t>
-        </is>
-      </c>
-      <c r="D5" s="3" t="n"/>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>E05</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>khanza__reg_periksa</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>Encounter</t>
-        </is>
-      </c>
-      <c r="D6" s="3" t="n"/>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>E06</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>khanza__diagnosa_pasien</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>Condition</t>
-        </is>
-      </c>
-      <c r="D7" s="3" t="n"/>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>E07</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>khanza__resep_obat</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>MedicationRequest</t>
-        </is>
-      </c>
-      <c r="D8" s="3" t="n"/>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>E08</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>khanza__resep_dokter</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>MedicationRequest</t>
-        </is>
-      </c>
-      <c r="D9" s="3" t="n"/>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>E09</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>khanza__databarang</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>Medication</t>
-        </is>
-      </c>
-      <c r="D10" s="3" t="n"/>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>E10</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>khanza__kamar_inap</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>Encounter</t>
-        </is>
-      </c>
-      <c r="D11" s="3" t="n"/>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>E11</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>khanza__penjab</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>Organization</t>
-        </is>
-      </c>
-      <c r="D12" s="3" t="n"/>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>E12</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>khanza__rujuk</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>ServiceRequest</t>
-        </is>
-      </c>
-      <c r="D13" s="3" t="n"/>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>E13</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>khanza__periksa_lab</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>DiagnosticReport</t>
-        </is>
-      </c>
-      <c r="D14" s="3" t="n"/>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>E14</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>khanza__detail_periksa_lab</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>Observation</t>
-        </is>
-      </c>
-      <c r="D15" s="3" t="n"/>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>E20</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>opensid__tweb_penduduk</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>Patient</t>
-        </is>
-      </c>
-      <c r="D16" s="3" t="n"/>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>E29</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>khanza__pasien_mati</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>Patient</t>
-        </is>
-      </c>
-      <c r="D17" s="3" t="n"/>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>E30</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>khanza__pasien_corona</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>Patient</t>
-        </is>
-      </c>
-      <c r="D18" s="3" t="n"/>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>E31</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>khanza__petugas</t>
-        </is>
-      </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>Practitioner</t>
-        </is>
-      </c>
-      <c r="D19" s="3" t="n"/>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>E32</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>khanza__perusahaan_pasien</t>
-        </is>
-      </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>Organization</t>
-        </is>
-      </c>
-      <c r="D20" s="3" t="n"/>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>E33</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>khanza__industrifarmasi</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>Organization</t>
-        </is>
-      </c>
-      <c r="D21" s="3" t="n"/>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>E34</t>
-        </is>
-      </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>khanza__datasuplier</t>
-        </is>
-      </c>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t>Organization</t>
-        </is>
-      </c>
-      <c r="D22" s="3" t="n"/>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>E35</t>
-        </is>
-      </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>khanza__bangsal</t>
-        </is>
-      </c>
-      <c r="C23" t="inlineStr">
-        <is>
-          <t>Location</t>
-        </is>
-      </c>
-      <c r="D23" s="3" t="n"/>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>E36</t>
-        </is>
-      </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>khanza__kamar</t>
-        </is>
-      </c>
-      <c r="C24" t="inlineStr">
-        <is>
-          <t>Location</t>
-        </is>
-      </c>
-      <c r="D24" s="3" t="n"/>
-    </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>E37</t>
-        </is>
-      </c>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t>khanza__ruang_ok</t>
-        </is>
-      </c>
-      <c r="C25" t="inlineStr">
-        <is>
-          <t>Location</t>
-        </is>
-      </c>
-      <c r="D25" s="3" t="n"/>
-    </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>E38</t>
-        </is>
-      </c>
-      <c r="B26" t="inlineStr">
-        <is>
-          <t>khanza__dpjp_ranap</t>
-        </is>
-      </c>
-      <c r="C26" t="inlineStr">
-        <is>
-          <t>Encounter</t>
-        </is>
-      </c>
-      <c r="D26" s="3" t="n"/>
-    </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>E39</t>
-        </is>
-      </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>khanza__resume_pasien</t>
-        </is>
-      </c>
-      <c r="C27" t="inlineStr">
-        <is>
-          <t>Condition</t>
-        </is>
-      </c>
-      <c r="D27" s="3" t="n"/>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>E40</t>
-        </is>
-      </c>
-      <c r="B28" t="inlineStr">
-        <is>
-          <t>khanza__pemeriksaan_ralan</t>
-        </is>
-      </c>
-      <c r="C28" t="inlineStr">
-        <is>
-          <t>Observation</t>
-        </is>
-      </c>
-      <c r="D28" s="3" t="n"/>
-    </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>E41</t>
-        </is>
-      </c>
-      <c r="B29" t="inlineStr">
-        <is>
-          <t>khanza__pemeriksaan_ranap</t>
-        </is>
-      </c>
-      <c r="C29" t="inlineStr">
-        <is>
-          <t>Observation</t>
-        </is>
-      </c>
-      <c r="D29" s="3" t="n"/>
-    </row>
-    <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>E42</t>
-        </is>
-      </c>
-      <c r="B30" t="inlineStr">
-        <is>
-          <t>khanza__catatan_observasi_igd</t>
-        </is>
-      </c>
-      <c r="C30" t="inlineStr">
-        <is>
-          <t>Observation</t>
-        </is>
-      </c>
-      <c r="D30" s="3" t="n"/>
-    </row>
-    <row r="31">
-      <c r="A31" t="inlineStr">
-        <is>
-          <t>E43</t>
-        </is>
-      </c>
-      <c r="B31" t="inlineStr">
-        <is>
-          <t>khanza__catatan_observasi_ranap</t>
-        </is>
-      </c>
-      <c r="C31" t="inlineStr">
-        <is>
-          <t>Observation</t>
-        </is>
-      </c>
-      <c r="D31" s="3" t="n"/>
-    </row>
-    <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t>E44</t>
-        </is>
-      </c>
-      <c r="B32" t="inlineStr">
-        <is>
-          <t>khanza__data_triase_igd</t>
-        </is>
-      </c>
-      <c r="C32" t="inlineStr">
-        <is>
-          <t>Observation</t>
-        </is>
-      </c>
-      <c r="D32" s="3" t="n"/>
-    </row>
-    <row r="33">
-      <c r="A33" t="inlineStr">
-        <is>
-          <t>E45</t>
-        </is>
-      </c>
-      <c r="B33" t="inlineStr">
-        <is>
-          <t>khanza__skrining_gizi</t>
-        </is>
-      </c>
-      <c r="C33" t="inlineStr">
-        <is>
-          <t>Observation</t>
-        </is>
-      </c>
-      <c r="D33" s="3" t="n"/>
-    </row>
-    <row r="34">
-      <c r="A34" t="inlineStr">
-        <is>
-          <t>E46</t>
-        </is>
-      </c>
-      <c r="B34" t="inlineStr">
-        <is>
-          <t>khanza__skrining_hipertensi</t>
-        </is>
-      </c>
-      <c r="C34" t="inlineStr">
-        <is>
-          <t>Observation</t>
-        </is>
-      </c>
-      <c r="D34" s="3" t="n"/>
-    </row>
-    <row r="35">
-      <c r="A35" t="inlineStr">
-        <is>
-          <t>E47</t>
-        </is>
-      </c>
-      <c r="B35" t="inlineStr">
-        <is>
-          <t>khanza__resep_dokter_racikan</t>
-        </is>
-      </c>
-      <c r="C35" t="inlineStr">
-        <is>
-          <t>MedicationRequest</t>
-        </is>
-      </c>
-      <c r="D35" s="3" t="n"/>
-    </row>
-    <row r="36">
-      <c r="A36" t="inlineStr">
-        <is>
-          <t>E48</t>
-        </is>
-      </c>
-      <c r="B36" t="inlineStr">
-        <is>
-          <t>khanza__resep_pulang</t>
-        </is>
-      </c>
-      <c r="C36" t="inlineStr">
-        <is>
-          <t>MedicationRequest</t>
-        </is>
-      </c>
-      <c r="D36" s="3" t="n"/>
-    </row>
-    <row r="37">
-      <c r="A37" t="inlineStr">
-        <is>
-          <t>E49</t>
-        </is>
-      </c>
-      <c r="B37" t="inlineStr">
-        <is>
-          <t>khanza__periksa_radiologi</t>
-        </is>
-      </c>
-      <c r="C37" t="inlineStr">
-        <is>
-          <t>DiagnosticReport</t>
-        </is>
-      </c>
-      <c r="D37" s="3" t="n"/>
-    </row>
-    <row r="38">
-      <c r="A38" t="inlineStr">
-        <is>
-          <t>E50</t>
-        </is>
-      </c>
-      <c r="B38" t="inlineStr">
-        <is>
-          <t>khanza__hasil_radiologi</t>
-        </is>
-      </c>
-      <c r="C38" t="inlineStr">
-        <is>
-          <t>DiagnosticReport</t>
-        </is>
-      </c>
-      <c r="D38" s="3" t="n"/>
-    </row>
-    <row r="39">
-      <c r="A39" t="inlineStr">
-        <is>
-          <t>E51</t>
-        </is>
-      </c>
-      <c r="B39" t="inlineStr">
-        <is>
-          <t>khanza__permintaan_lab</t>
-        </is>
-      </c>
-      <c r="C39" t="inlineStr">
-        <is>
-          <t>ServiceRequest</t>
-        </is>
-      </c>
-      <c r="D39" s="3" t="n"/>
-    </row>
-    <row r="40">
-      <c r="A40" t="inlineStr">
-        <is>
-          <t>E52</t>
-        </is>
-      </c>
-      <c r="B40" t="inlineStr">
-        <is>
-          <t>khanza__permintaan_radiologi</t>
-        </is>
-      </c>
-      <c r="C40" t="inlineStr">
-        <is>
-          <t>ServiceRequest</t>
-        </is>
-      </c>
-      <c r="D40" s="3" t="n"/>
-    </row>
-    <row r="41">
-      <c r="A41" t="inlineStr">
-        <is>
-          <t>E53</t>
-        </is>
-      </c>
-      <c r="B41" t="inlineStr">
-        <is>
-          <t>khanza__rujukan_internal_poli</t>
-        </is>
-      </c>
-      <c r="C41" t="inlineStr">
-        <is>
-          <t>ServiceRequest</t>
-        </is>
-      </c>
-      <c r="D41" s="3" t="n"/>
-    </row>
-    <row r="42">
-      <c r="A42" t="inlineStr">
-        <is>
-          <t>E54</t>
-        </is>
-      </c>
-      <c r="B42" t="inlineStr">
-        <is>
-          <t>khanza__rujuk_masuk</t>
-        </is>
-      </c>
-      <c r="C42" t="inlineStr">
-        <is>
-          <t>ServiceRequest</t>
-        </is>
-      </c>
-      <c r="D42" s="3" t="n"/>
-    </row>
-    <row r="43">
-      <c r="A43" t="inlineStr">
-        <is>
-          <t>C01</t>
-        </is>
-      </c>
-      <c r="B43" t="inlineStr">
-        <is>
-          <t>rmpuskesmas__tb_pasien</t>
-        </is>
-      </c>
-      <c r="C43" t="inlineStr">
-        <is>
-          <t>Patient</t>
-        </is>
-      </c>
-      <c r="D43" s="3" t="n"/>
-    </row>
-    <row r="44">
-      <c r="A44" t="inlineStr">
-        <is>
-          <t>C02</t>
-        </is>
-      </c>
-      <c r="B44" t="inlineStr">
-        <is>
-          <t>rmpuskesmas__tb_rekam_medis</t>
-        </is>
-      </c>
-      <c r="C44" t="inlineStr">
-        <is>
-          <t>Encounter</t>
-        </is>
-      </c>
-      <c r="D44" s="3" t="n"/>
-    </row>
-    <row r="45">
-      <c r="A45" t="inlineStr">
-        <is>
-          <t>C03</t>
-        </is>
-      </c>
-      <c r="B45" t="inlineStr">
-        <is>
-          <t>rmpuskesmas__tb_rujuk</t>
-        </is>
-      </c>
-      <c r="C45" t="inlineStr">
-        <is>
-          <t>ServiceRequest</t>
-        </is>
-      </c>
-      <c r="D45" s="3" t="n"/>
-    </row>
-    <row r="46">
-      <c r="A46" t="inlineStr">
-        <is>
-          <t>C04</t>
-        </is>
-      </c>
-      <c r="B46" t="inlineStr">
-        <is>
-          <t>rmpuskesmas__tb_resep</t>
-        </is>
-      </c>
-      <c r="C46" t="inlineStr">
-        <is>
-          <t>MedicationRequest</t>
-        </is>
-      </c>
-      <c r="D46" s="3" t="n"/>
-    </row>
-    <row r="47">
-      <c r="A47" t="inlineStr">
-        <is>
-          <t>C05</t>
-        </is>
-      </c>
-      <c r="B47" t="inlineStr">
-        <is>
-          <t>rmpuskesmas__tb_dokter</t>
-        </is>
-      </c>
-      <c r="C47" t="inlineStr">
-        <is>
-          <t>Practitioner</t>
-        </is>
-      </c>
-      <c r="D47" s="3" t="n"/>
-    </row>
-    <row r="48">
-      <c r="A48" t="inlineStr">
-        <is>
-          <t>C06</t>
-        </is>
-      </c>
-      <c r="B48" t="inlineStr">
-        <is>
-          <t>sipuskesmas__polis</t>
-        </is>
-      </c>
-      <c r="C48" t="inlineStr">
-        <is>
-          <t>Location</t>
-        </is>
-      </c>
-      <c r="D48" s="3" t="n"/>
-    </row>
-    <row r="49">
-      <c r="A49" t="inlineStr">
-        <is>
-          <t>C07</t>
-        </is>
-      </c>
-      <c r="B49" t="inlineStr">
-        <is>
-          <t>sipuskesmas__tenaga_kesehatans</t>
-        </is>
-      </c>
-      <c r="C49" t="inlineStr">
-        <is>
-          <t>Practitioner</t>
-        </is>
-      </c>
-      <c r="D49" s="3" t="n"/>
-    </row>
-    <row r="50">
-      <c r="A50" t="inlineStr">
-        <is>
-          <t>C08</t>
-        </is>
-      </c>
-      <c r="B50" t="inlineStr">
-        <is>
-          <t>sipuskesmas__antrians</t>
-        </is>
-      </c>
-      <c r="C50" t="inlineStr">
-        <is>
-          <t>Encounter</t>
-        </is>
-      </c>
-      <c r="D50" s="3" t="n"/>
-    </row>
-    <row r="51">
-      <c r="A51" t="inlineStr">
-        <is>
-          <t>C09</t>
-        </is>
-      </c>
-      <c r="B51" t="inlineStr">
-        <is>
-          <t>cirekammedis__dokter</t>
-        </is>
-      </c>
-      <c r="C51" t="inlineStr">
-        <is>
-          <t>Practitioner</t>
-        </is>
-      </c>
-      <c r="D51" s="3" t="n"/>
-    </row>
-    <row r="52">
-      <c r="A52" t="inlineStr">
-        <is>
-          <t>C10</t>
-        </is>
-      </c>
-      <c r="B52" t="inlineStr">
-        <is>
-          <t>cirekammedis__obat</t>
-        </is>
-      </c>
-      <c r="C52" t="inlineStr">
-        <is>
-          <t>Medication</t>
-        </is>
-      </c>
-      <c r="D52" s="3" t="n"/>
-    </row>
-    <row r="53">
-      <c r="A53" t="inlineStr">
-        <is>
-          <t>C11</t>
-        </is>
-      </c>
-      <c r="B53" t="inlineStr">
-        <is>
-          <t>cirekammedis__pasien</t>
-        </is>
-      </c>
-      <c r="C53" t="inlineStr">
-        <is>
-          <t>Patient</t>
-        </is>
-      </c>
-      <c r="D53" s="3" t="n"/>
-    </row>
-    <row r="54">
-      <c r="A54" t="inlineStr">
-        <is>
-          <t>C12</t>
-        </is>
-      </c>
-      <c r="B54" t="inlineStr">
-        <is>
-          <t>cirekammedis__poliklinik</t>
-        </is>
-      </c>
-      <c r="C54" t="inlineStr">
-        <is>
-          <t>Location</t>
-        </is>
-      </c>
-      <c r="D54" s="3" t="n"/>
-    </row>
-    <row r="55">
-      <c r="A55" t="inlineStr">
-        <is>
-          <t>C13</t>
-        </is>
-      </c>
-      <c r="B55" t="inlineStr">
-        <is>
-          <t>cirekammedis__rekam_medis</t>
-        </is>
-      </c>
-      <c r="C55" t="inlineStr">
-        <is>
-          <t>Encounter</t>
-        </is>
-      </c>
-      <c r="D55" s="3" t="n"/>
-    </row>
-    <row r="56">
-      <c r="A56" t="inlineStr">
-        <is>
-          <t>C14</t>
-        </is>
-      </c>
-      <c r="B56" t="inlineStr">
-        <is>
-          <t>cirekammedis__rm_obat</t>
-        </is>
-      </c>
-      <c r="C56" t="inlineStr">
-        <is>
-          <t>MedicationRequest</t>
-        </is>
-      </c>
-      <c r="D56" s="3" t="n"/>
-    </row>
-    <row r="57">
-      <c r="A57" t="inlineStr">
-        <is>
-          <t>C15</t>
-        </is>
-      </c>
-      <c r="B57" t="inlineStr">
-        <is>
-          <t>sipograf__t_anak</t>
-        </is>
-      </c>
-      <c r="C57" t="inlineStr">
-        <is>
-          <t>Patient</t>
-        </is>
-      </c>
-      <c r="D57" s="3" t="n"/>
-    </row>
-    <row r="58">
-      <c r="A58" t="inlineStr">
-        <is>
-          <t>C16</t>
-        </is>
-      </c>
-      <c r="B58" t="inlineStr">
-        <is>
-          <t>sipograf__t_penimbangan</t>
-        </is>
-      </c>
-      <c r="C58" t="inlineStr">
-        <is>
-          <t>Observation</t>
-        </is>
-      </c>
-      <c r="D58" s="3" t="n"/>
-    </row>
-    <row r="59">
-      <c r="A59" t="inlineStr">
-        <is>
-          <t>C17</t>
-        </is>
-      </c>
-      <c r="B59" t="inlineStr">
-        <is>
-          <t>epuskesmas__obat</t>
-        </is>
-      </c>
-      <c r="C59" t="inlineStr">
-        <is>
-          <t>Medication</t>
-        </is>
-      </c>
-      <c r="D59" s="3" t="n"/>
-    </row>
-    <row r="60">
-      <c r="A60" t="inlineStr">
-        <is>
-          <t>C18</t>
-        </is>
-      </c>
-      <c r="B60" t="inlineStr">
-        <is>
-          <t>opensid__posyandu</t>
-        </is>
-      </c>
-      <c r="C60" t="inlineStr">
-        <is>
-          <t>Organization</t>
-        </is>
-      </c>
-      <c r="D60" s="3" t="n"/>
-    </row>
-  </sheetData>
-  <dataValidations count="1">
-    <dataValidation sqref="D2 D3 D4 D5 D6 D7 D8 D9 D10 D11 D12 D13 D14 D15 D16 D17 D18 D19 D20 D21 D22 D23 D24 D25 D26 D27 D28 D29 D30 D31 D32 D33 D34 D35 D36 D37 D38 D39 D40 D41 D42 D43 D44 D45 D46 D47 D48 D49 D50 D51 D52 D53 D54 D55 D56 D57 D58 D59 D60" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"ya,tidak"</formula1>
-    </dataValidation>
-  </dataValidations>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -24484,7 +23106,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -24961,7 +23583,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -25234,7 +23856,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -25677,7 +24299,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -26494,7 +25116,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -26903,7 +25525,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -27667,4 +26289,260 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C14"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="32" customWidth="1" min="1" max="1"/>
+    <col width="90" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>elemen</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>tipe</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>deskripsi (FHIR short)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>identifier</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Identifier</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Business identifier for this medication</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>CodeableConcept</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Codes that identify this medication</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>status</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>active | inactive | entered-in-error</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>manufacturer</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Reference</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Manufacturer of the item</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>form</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>CodeableConcept</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>powder | tablets | capsule +</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>amount</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Ratio</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Amount of drug in package</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>ingredient</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>BackboneElement</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Active or inactive ingredient</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>ingredient.item[x]</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>CodeableConcept|Reference</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>The actual ingredient or content</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>ingredient.isActive</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>boolean</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Active ingredient indicator</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>ingredient.strength</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Ratio</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Quantity of ingredient present</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>batch</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>BackboneElement</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Details about packaged medications</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>batch.lotNumber</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Identifier assigned to batch</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>batch.expirationDate</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>dateTime</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>When batch will expire</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>